<commit_message>
chore(funnel): commit pending funnel work from earlier sessions
Work that piled up uncommitted across previous sessions:
- ChatChi (chai-*): hard-paywall/add-on/web-paywall passes, images and
  build scripts for roleplay, short-drama, named-character, dream-girl,
  ai-boyfriend/girlfriend, companion, romance-stories; QA test folders
- CoinIdentify (scanner/coinin*): rebrand, plans, images
- Starlyn (nebula/*, starlyn): monetization + add-on updates
- ai-photo-video, learning, mental-health, authenticator, testlibrary
  brief/demo updates; funnel-content-writer skill references
- FunnelFox exports/uploads, pricing and competitor research sheets,
  smoke_demo tool

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/funnel/funnel-testing/chat-ai-character/ChatChi-ALL_UI_Bug_Report_06102026.xlsx
+++ b/funnel/funnel-testing/chat-ai-character/ChatChi-ALL_UI_Bug_Report_06102026.xlsx
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J75"/>
+  <dimension ref="A1:K75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1105,6 +1105,7 @@
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1158,6 +1159,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Dev note (07/10)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="n">
@@ -1205,7 +1211,12 @@
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>Màn cao &lt;=700px: thu nhỏ herorow (zoom .7) và wheel còn 132px (3 dòng); ở 375x667 box năm hiện trọn trong first view (đáy box 485px &lt; vùng scroll 500px). Màn lớn không đổi.</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1266,12 @@
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not a bug</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>Thiết kế cố ý: mỗi archetype có hashtag ngắn riêng (C[k].tag: #MorallyGrey, #Grumpy, #GoldenRetriever...), tên đầy đủ đã hiện ở chip paywall và màn chọn. Spec chỉ ghi 'archetype tag', không bắt buộc tên đầy đủ; tên đầy đủ dài sẽ tràn plate. Giữ nguyên, PM/Designer có thể đổi sau.</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1321,12 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>Bỏ emoji trang trí 190px trong nền chat (.cbg span); nền chỉ còn ảnh scene mờ. Hết lỗi ở he_texts_first, he_remembers, good_morning_texts (auto-check sạch).</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1376,12 @@
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>'Terms' và 'Privacy Policy' giờ là thẻ &lt;a&gt; thật (CONFIG.legal URL, target=_blank), gạch chân, chữ 13px, vùng bấm cao 42px. Đồng thời nâng legal link chung (Intro 1, sale, upsell) lên 13px, gạch chân rõ hơn, cao 44px.</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1431,12 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>Top bar khi cuộn và sticky bottom bar dùng nền đặc var(--bg), bỏ trong suốt/blur. Thêm: sticky bar giờ hiện bất cứ khi nào CTA của plan block không nằm trong màn hình (trước đây chỉ cần plan block lọt vào là ẩn, nên ở 430x932 first view không thấy CTA).</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1486,12 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>Link support gạch chân, chữ 13px, vùng bấm 136x44px (trước 114x15).</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1541,12 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>Footer 'No thanks' + Terms/Privacy ở sale_m1/m3/y12, sale_lifetime, upsell_lifetime chuyển vào vùng cuộn, nằm sau card (margin-top:auto nên màn lớn vẫn ở đáy). 375x667: renewal line và AI disclosure hiện đủ ở first view, không bị che.</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1596,12 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>Xoá hẳn màn last_chance_offer: view, SCREENS entry, OFFER_ID, hàm offer*, action offerbuy/offerno, CONFIG.offer có {{offer_*}} và CSS liên quan. Decline vẫn về paywall (DECLINE_FALLBACK). ff_engine_build build OK, checkout không đổi; #s=99 không còn màn nào.</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1651,12 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>Thay bằng badge chính thức: SVG 'Download on the App Store' (đen) tải từ developer.apple.com và PNG 'GET IT ON Google Play' từ play.google.com (cắt viền trong suốt), nhúng data URI, cao 46px. Vẫn gọi openApp().</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1706,12 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>Màn thấp (≤700px) thu nhỏ hàng hero (card + lock-screen scale ~0.8, cao 214→168px) nên box year wheel hiện đủ 3 dòng ở first view 375×667; 430×932 không đổi.</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1761,12 @@
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>Dấu ? + chữ "Tap a hair colour" nằm trong ô nền đặc có viền, nét sketch không còn đè lên chữ (cả 2 viewport).</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1816,12 @@
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="inlineStr">
+        <is>
+          <t>Đổi her_age sang 4 option xếp dọc đúng spec #3 ("Four stacked pills"); vẫn vừa first view 375×667, CTA không bị đẩy.</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1871,12 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K14" s="12" t="inlineStr">
+        <is>
+          <t>Preview card nhỏ (&lt;110px, màn names và personality) ẩn chip/ribbon overlay; thông tin đã có ở danh sách bên cạnh nên portrait thấy rõ. Card cỡ thường ở màn 2-7 giữ nguyên.</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1926,12 @@
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>Verify bằng click thật: bug có thật khi chọn hair 'Other' (field trống, card hiện 'Luna'). Màn names giờ prefill tên gợi ý trùng tên trên card nếu user chưa tự sửa; chọn màu thường vẫn prefill như cũ (Chloe...).</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1981,12 @@
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K16" s="12" t="inlineStr">
+        <is>
+          <t>Avatar + "Ivy · Cozy" chuyển sang góc trên bên phải đúng spec #10.</t>
         </is>
       </c>
     </row>
@@ -1955,7 +2036,12 @@
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K17" s="12" t="inlineStr">
+        <is>
+          <t>Cùng fix với #13: card nhỏ ở personality không còn chip overlay nên không còn chồng/cắt chữ, portrait thấy rõ.</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2091,12 @@
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K18" s="12" t="inlineStr">
+        <is>
+          <t>Sticky bar (giá hôm nay $119.99 + Continue) giờ hiện bất cứ khi nào CTA của plan block chưa nằm trọn trong khung hình, kể cả first view 430×932 và 375×667 (theo mẫu boyfriend). Nền đặc, lps có padding đáy nên không che nội dung cuối; top bar cũng nền đặc.</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2146,12 @@
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>Link support gạch chân, cao 44px (padding), chữ 13px; Terms/Privacy cũng tăng lên 13px, màu sáng hơn, gạch chân rõ, tap 44px. qa_capture không còn cảnh báo tap target.</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2201,12 @@
       </c>
       <c r="J20" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K20" s="12" t="inlineStr">
+        <is>
+          <t>Thay pill chữ bằng mark SVG inline: Apple Pay (logo táo + Pay, nền đen), Google Pay (G 4 màu), VISA (wordmark xanh), Mastercard (2 vòng tròn đỏ/vàng), PayPal (2 tông xanh). Artwork vẽ lại gần bản gốc; nếu Designer có file brand chính thức có thể thay sau.</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2256,12 @@
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K21" s="12" t="inlineStr">
+        <is>
+          <t>Màn sale_m1/m3/y12/lifetime và upsell giờ cuộn cả trang, footer (No thanks + Terms/Privacy) nằm sau card thay vì cố định; renewal line và dòng AI disclosure hiện đủ ở 375×667. Top bar sticky nền đặc.</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2311,12 @@
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K22" s="12" t="inlineStr">
+        <is>
+          <t>Xoá hẳn màn last_chance_offer (view, SCREENS[22], OFFER_ID, CONFIG.offer với token {{offer_*}}, handler offerbuy/offerno, CSS thừa). ff_engine_build vẫn build OK, INDEX/checkout screens không đổi.</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2366,12 @@
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K23" s="12" t="inlineStr">
+        <is>
+          <t>Dùng badge chính thức: Apple "Download on the App Store" (SVG đen từ Apple Marketing Tools) và Google Play "GET IT ON" (PNG từ play.google.com), nhúng data URI; vẫn gọi openApp(), link web2app/web2web không đổi.</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2421,12 @@
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K24" s="12" t="inlineStr">
+        <is>
+          <t>Bỏ căn giữa dọc ở Intro 4 (friend_not_therapist) và Intro 8 (memory_control): headline nằm ngay dưới progress bar như Intro 2, 3, 5, 6, 7 ở cả 375 và 430.</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2476,12 @@
       </c>
       <c r="J25" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>Màn thấp (&lt;=700px): card personality thấp lại (122-&gt;100px) và hero Meet giảm (276-&gt;246px), nên hàng He/She/They/Surprise me và hàng Or talk with Noor/Ben hiển thị đủ ở 375x667. Thêm fade ở mép dưới vùng cuộn mỗi khi màn còn nội dung bên dưới.</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2531,12 @@
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K26" s="12" t="inlineStr">
+        <is>
+          <t>Bar bị trễ do transition 0.3s ease trong khi số % nhảy mỗi 42ms. Đổi sang 40ms linear: độ lệch số/bar tối đa 23% -&gt; ~5% (1 tick).</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2586,12 @@
       </c>
       <c r="J27" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>Terms và Privacy Policy ở màn email giờ là thẻ &lt;a&gt; thật tới CONFIG.legal (target=_blank), gạch chân, chữ sáng hơn, 13px, vùng bấm cao 43px. Legal links ở paywall/sale/upsell/intro 1 cũng nâng lên 13px, màu t2, gạch chân rõ hơn; support@chatchi.co 13px.</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2641,12 @@
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K28" s="12" t="inlineStr">
+        <is>
+          <t>Sticky bar (ChatChi Plus · 12 months / Due today $119.99 / Continue) và mini Continue giờ hiện khi không có nút CTA của plan block nào hiện đủ trên màn (trừ vùng header sticky), nên first view ở 430x932 và 375x667 đều có giá + CTA. Nền sticky bar và top bar đổi sang màu đặc; footer vẫn có padding đáy nên sticky không che nội dung cuối.</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2696,12 @@
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K29" s="12" t="inlineStr">
+        <is>
+          <t>Footer No thanks + Terms/Privacy của các màn sale (và upsell) chuyển vào trong vùng cuộn (flow, margin-top:auto), không còn cố định che nội dung: dòng ChatChi is AI, not therapy hiện ngay first view ở 375x667 cho sale_m1/m3/y12.</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2751,12 @@
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K30" s="12" t="inlineStr">
+        <is>
+          <t>Card Bonus companion dùng avatar 'companion mới' (vòng viền nét đứt, icon người, badge +) thay cho ảnh Sam, đúng nghĩa là tạo companion thứ hai. Brief cập nhật theo.</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2806,12 @@
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K31" s="12" t="inlineStr">
+        <is>
+          <t>Xoá hẳn màn last_chance_offer (view, SCREENS[20], OFFER_ID, timer, action offerbuy/offerno, CSS) và token {{offer_*}} khỏi CONFIG (offer:{enabled:false}). Screen không tồn tại -&gt; về paywall. ff_engine_build.py vẫn build OK (offerId=0), ids và checkout screens không đổi.</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2861,12 @@
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>Dòng 18+ + Terms/Privacy chuyển xuống footer ghim đáy màn Intro 1, luôn thấy ở first view 375x667 trước khi tap card (bottom 649px &lt; 667). Brief #1 đã cập nhật.</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2916,12 @@
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K33" s="12" t="inlineStr">
+        <is>
+          <t>Mọi link Terms/Privacy (Intro 1, sale, lifetime, upsell, footer paywall) + support@chatchi.co (giờ là link mailto): &lt;a&gt; thật target=_blank, chữ 13px, gạch chân màu hồng nhạt, vùng bấm cao 40px (đo 94x40 / 98x40 / 136x40).</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2971,12 @@
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not a bug</t>
+        </is>
+      </c>
+      <c r="K34" s="12" t="inlineStr">
+        <is>
+          <t>Quiz có đúng 9 bước (màn 2-10) nên 9 segment là đúng; lỗi nằm ở brief, đã sửa funnel-content.md #2 thành 9-segment.</t>
         </is>
       </c>
     </row>
@@ -2855,7 +3026,12 @@
       </c>
       <c r="J35" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K35" s="12" t="inlineStr">
+        <is>
+          <t>Gen lại img/fig-athletic.jpg (gemini-3.1-flash-image, prompt bỏ gương, một người trong khung); ảnh mới chỉ còn 1 nhân vật.</t>
         </is>
       </c>
     </row>
@@ -2905,7 +3081,12 @@
       </c>
       <c r="J36" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>Sticky bar (gói + giá today + Get my AI girl) hiện từ first view khi không có CTA của plan block trên màn (cả 375x667 và 430x932), ẩn khi CTA plan block hiện; nền đặc; footer padding-bottom 140px để không che dòng cuối.</t>
         </is>
       </c>
     </row>
@@ -2955,7 +3136,12 @@
       </c>
       <c r="J37" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>Gen 16 portrait her-&lt;ethnicity&gt;-&lt;hair&gt;.jpg; herImg() chọn ảnh theo ethnicity + hair (ảnh card ethnicity khi tóc trùng mặc định hoặc No preference). Áp dụng cho paywall, email, loader, chat, sale, upsell. Brief #13 cập nhật.</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3191,12 @@
       </c>
       <c r="J38" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K38" s="12" t="inlineStr">
+        <is>
+          <t>Top bar sale_m1/m3/y12/lifetime/upsell: nền đặc var(--bg) + divider như Paywall 1; top bar paywall và sticky bar cũng bỏ nền trong suốt/blur.</t>
         </is>
       </c>
     </row>
@@ -3055,7 +3246,12 @@
       </c>
       <c r="J39" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K39" s="12" t="inlineStr">
+        <is>
+          <t>Thay bằng artwork chính thức (SVG 'Download on the App Store' đen của Apple, PNG 'GET IT ON Google Play' của Google) nhúng data URI, cao 44px, vẫn gọi openApp().</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3301,12 @@
       </c>
       <c r="J40" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K40" s="12" t="inlineStr">
+        <is>
+          <t>Xoá hẳn màn last_chance_offer (V[99], SCREENS, OFFER_ID, CONFIG.offer với token {{offer_*}}, handler offerbuy/offerno, CSS). ff_engine_build.py vẫn build OK (không có offer), #s=99 không còn mở được.</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3356,12 @@
       </c>
       <c r="J41" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K41" s="12" t="inlineStr">
+        <is>
+          <t>Link Terms/Privacy ở mọi màn (hook, email_gate, paywall footer, sale, upsell) là thẻ &lt;a&gt; thật (CONFIG.legal, target=_blank), màu link hồng + gạch chân, 13–13.5px, cao 40px (đo: Terms 50x40, Terms of Use 94x40). Email gate tách link xuống dòng riêng.</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3411,12 @@
       </c>
       <c r="J42" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K42" s="12" t="inlineStr">
+        <is>
+          <t>Sticky bar ("12 months plan · $119.99 today" + Continue with Lena) hiện ngay first view ở 375x667 và 430x932, chỉ ẩn khi CTA của plan block đang trên màn; nền đặc; footer có padding đáy nên bar không che nội dung cuối.</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3466,12 @@
       </c>
       <c r="J43" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K43" s="12" t="inlineStr">
+        <is>
+          <t>support@chatchi.co ở footer giờ là link mailto, cùng style link và tap target 40px như Terms/Privacy.</t>
         </is>
       </c>
     </row>
@@ -3305,7 +3521,12 @@
       </c>
       <c r="J44" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K44" s="12" t="inlineStr">
+        <is>
+          <t>Top bar của sale_m1/m3/y12/lifetime và upsell_lifetime đổi sang nền đặc + divider như paywall; top bar paywall và sticky bar cũng bỏ nền trong suốt/blur, dùng nền đặc.</t>
         </is>
       </c>
     </row>
@@ -3355,7 +3576,12 @@
       </c>
       <c r="J45" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K45" s="12" t="inlineStr">
+        <is>
+          <t>Thay bằng artwork chính thức: SVG badge "Download on the App Store" tải từ developer.apple.com và PNG badge "GET IT ON Google Play" từ play.google.com, nhúng data URI; vẫn gọi openApp().</t>
         </is>
       </c>
     </row>
@@ -3405,7 +3631,12 @@
       </c>
       <c r="J46" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K46" s="12" t="inlineStr">
+        <is>
+          <t>Xoá hẳn màn last_chance_offer (OFFER_ID 99, view, SCREENS, handler offerbuy/offerno, CONFIG.offer có {{offer_*}}). ff_engine_build.py vẫn build OK (offerId=0, không có offer); checkout không đổi.</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3686,12 @@
       </c>
       <c r="J47" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K47" s="12" t="inlineStr">
+        <is>
+          <t>Căn giữa theo chiều dọc cụm logo/tag/headline/fan card; màn cao (&gt;=780px) phóng to card 138x208 và giãn fan, nên không còn nửa màn trống ở 430x932; 375x667 cân đối.</t>
         </is>
       </c>
     </row>
@@ -3505,7 +3741,12 @@
       </c>
       <c r="J48" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K48" s="12" t="inlineStr">
+        <is>
+          <t>Thêm tag pill "AI roleplay" ngay dưới logo ChatChi đúng Spec #1.</t>
         </is>
       </c>
     </row>
@@ -3555,7 +3796,12 @@
       </c>
       <c r="J49" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K49" s="12" t="inlineStr">
+        <is>
+          <t>Mọi link legal (age gate, trust, email, footer paywall gồm support@chatchi.co, sale/lifetime/upsell) là &lt;a&gt; thật tới CONFIG.legal (target=_blank), gạch chân màu chữ sáng, cỡ 13px, cao 40px nhờ padding (đo lại 375x667: 94x40, 98x40, 136x40...).</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3851,12 @@
       </c>
       <c r="J50" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K50" s="12" t="inlineStr">
+        <is>
+          <t>Thêm nền ảnh storybook (hook.jpg) làm mờ + tối phía sau và box surface bo góc chứa Month/Year select + legal, đúng Spec #2.</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3906,12 @@
       </c>
       <c r="J51" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K51" s="12" t="inlineStr">
+        <is>
+          <t>Role: icon line (khiên/kiếm chéo/la bàn/bút) tô màu accent của genre thay emoji. Setting: hàng ngang 3 card cao, mỗi card một ảnh cảnh riêng, tên serif. Tone: 3 card lớn có thumbnail cảnh genre theo mood (sáng / tối / ánh vàng) + mô tả ngắn.</t>
         </is>
       </c>
     </row>
@@ -3705,7 +3961,12 @@
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K52" s="12" t="inlineStr">
+        <is>
+          <t>Sinh 15 ảnh cảnh riêng (set-&lt;genre&gt;-&lt;n&gt;.jpg, gemini-3.1-flash-image, cùng style painterly): Ember Keep / Whisperwood / Drowned Harbour... mỗi setting một ảnh, cho cả 5 genre; ảnh setting cũng dùng cho scene card ở cliffhanger.</t>
         </is>
       </c>
     </row>
@@ -3755,7 +4016,12 @@
       </c>
       <c r="J53" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K53" s="12" t="inlineStr">
+        <is>
+          <t>Sinh 15 portrait companion (comp-&lt;genre&gt;-&lt;n&gt;.jpg, người lớn 25+, mặc đủ, không chữ) và thay emoji ở companion, character_name, cover story_reveal, header chat, hero + mock chat paywall, sale/lifetime/upsell; scene card cliffhanger dùng ảnh setting thay emoji rồng. Emoji chỉ còn làm fallback dưới ảnh.</t>
         </is>
       </c>
     </row>
@@ -3805,7 +4071,12 @@
       </c>
       <c r="J54" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K54" s="12" t="inlineStr">
+        <is>
+          <t>Reproduce bằng luồng click thật (story_reveal -&gt; chọn action -&gt; scene_turn_2): toast đè header. Đổi thành note có icon sổ tay trượt vào trong thread ngay dưới câu trả lời cuối, không còn overlay header (top 361px &gt; header 59px).</t>
         </is>
       </c>
     </row>
@@ -3855,7 +4126,12 @@
       </c>
       <c r="J55" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K55" s="12" t="inlineStr">
+        <is>
+          <t>Làm theo mẫu chai-ai-boyfriend: sticky bar (tên plan + giá hôm nay + Continue + dòng renew) hiện ngay first view ở 375x667 và 430x932, chỉ ẩn khi CTA của plan block hoặc footer đang trên màn; nền đặc + viền trên; footer thêm padding đáy. Cập nhật assertion tương ứng trong qa-chai-roleplay.mjs.</t>
         </is>
       </c>
     </row>
@@ -3905,7 +4181,12 @@
       </c>
       <c r="J56" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K56" s="12" t="inlineStr">
+        <is>
+          <t>Top bar (logo + X) của sale_m1/m3/y12, sale_lifetime, upsell_lifetime đổi sang nền đặc + divider như Paywall 1; text cuộn không còn lộ dưới logo. Các màn này không có footer fixed nên dòng renew/AI disclosure không bị che.</t>
         </is>
       </c>
     </row>
@@ -3955,7 +4236,12 @@
       </c>
       <c r="J57" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K57" s="12" t="inlineStr">
+        <is>
+          <t>Google Play: dùng đúng artwork badge chính thức của Google (en_badge_web_generic, crop, nhúng data URI). App Store: không tải được từ apple.com (DNS bị chặn) nên vẽ SVG inline theo badge đen chính thức (logo Apple + "Download on the / App Store", viền #A6A6A6). Cao 44px, vẫn gọi openApp().</t>
         </is>
       </c>
     </row>
@@ -4005,7 +4291,12 @@
       </c>
       <c r="J58" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K58" s="12" t="inlineStr">
+        <is>
+          <t>Màn thấp (≤700px): hero zoom .66, year wheel cao 132px. Ở 375×667 hint hiện đủ trên CTA, .scr không còn phải cuộn (494/494).</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4346,12 @@
       </c>
       <c r="J59" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K59" s="12" t="inlineStr">
+        <is>
+          <t>Card trope luôn chỉ hiện eyebrow ngắn "CHATCHI" (ẩn " · A romance story"). Không còn đè emoji, 2 viewport giống nhau.</t>
         </is>
       </c>
     </row>
@@ -4105,7 +4401,12 @@
       </c>
       <c r="J60" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K60" s="12" t="inlineStr">
+        <is>
+          <t>"Surprise me" giờ hiện ảnh ghép hai lead (nữ + nam) của trope, blend mềm, không trùng ảnh "A man"/"A woman". Dùng lại ảnh có sẵn, không gen ảnh mới.</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4456,12 @@
       </c>
       <c r="J61" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K61" s="12" t="inlineStr">
+        <is>
+          <t>Đã tái hiện: cuộn .scr làm Chrome vẽ thiếu nửa dưới cover 3D. Đưa sách 3D ra ngoài vùng cuộn, thu nhỏ sách trên màn &lt;720px (158×218). Cover đủ title/portrait/tag cả khi cuộn, animation mở bìa vẫn đúng.</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4511,12 @@
       </c>
       <c r="J62" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K62" s="12" t="inlineStr">
+        <is>
+          <t>Nút 1x/mute: kích thước 38×32, vùng bấm ::before mở rộng thành 44×44. Nút play/pause: vùng bấm 44×44. Label "Narrated by … · Warm" không bị cắt. Áp dụng cho mọi màn chat (10/11/15/16/17).</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4566,12 @@
       </c>
       <c r="J63" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not a bug</t>
+        </is>
+      </c>
+      <c r="K63" s="12" t="inlineStr">
+        <is>
+          <t>Ảnh QA chụp lúc 1.2s, khi card đang flip. Chụp lại ở 3.5s: card đã lật có illustration, caption đúng "Chapter card 1/12 saved to your library".</t>
         </is>
       </c>
     </row>
@@ -4305,7 +4621,12 @@
       </c>
       <c r="J64" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K64" s="12" t="inlineStr">
+        <is>
+          <t>Footer (No thanks + Terms/Privacy) của 4 màn sale (m1/m3/y12/lifetime) giờ nằm trong vùng cuộn, không pinned. Ở 375×667 và 360×640, dòng renewal và AI disclosure đọc đủ, đóng vẫn bằng nút X trên top bar.</t>
         </is>
       </c>
     </row>
@@ -4355,7 +4676,12 @@
       </c>
       <c r="J65" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K65" s="12" t="inlineStr">
+        <is>
+          <t>Xoá màn last_chance_offer (view, SCREENS[99], timer, action offerbuy/offerno, CSS) và token {{offer_*}} khỏi CONFIG.offer (giữ {enabled:false}). Giữ hằng OFFER_ID cho ff_engine_build. Debug jump tới 99 giờ bị bỏ qua. FF build OK.</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4731,12 @@
       </c>
       <c r="J66" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K66" s="12" t="inlineStr">
+        <is>
+          <t>Link Terms/Privacy/support@chatchi.co ở age_gate, save_progress, paywall, sale, upsell: cỡ chữ 13px, màu link + gạch chân, vùng bấm cao 40px (trước 14px). Vẫn là &lt;a&gt; tới CONFIG.legal, target=_blank.</t>
         </is>
       </c>
     </row>
@@ -4455,7 +4786,12 @@
       </c>
       <c r="J67" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K67" s="12" t="inlineStr">
+        <is>
+          <t>Gen lại series-thriller.jpg (gemini-3.1-flash-image) với Nora là nữ thám tử mặc trench coat; poster ở Intro 1, Intro 3, các slide tập Night Shift đều khớp lead.</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4841,12 @@
       </c>
       <c r="J68" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K68" s="12" t="inlineStr">
+        <is>
+          <t>Top bar màn your_name đổi thành "Your name"; series_pick giữ "Your series".</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4896,12 @@
       </c>
       <c r="J69" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K69" s="12" t="inlineStr">
+        <is>
+          <t>Gen 3 portrait lead (Leo, Nora, Alden – người lớn, mặc đồ, không chữ) vào img/lead-*.jpg; dùng ở your_name, cliffhanger, header chat, quote paywall, thẻ sale/upsell. Emoji chỉ còn là fallback khi ảnh lỗi.</t>
         </is>
       </c>
     </row>
@@ -4605,7 +4951,12 @@
       </c>
       <c r="J70" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K70" s="12" t="inlineStr">
+        <is>
+          <t>Brief #6 quy định cùng story frame, grade tối hơn: thêm grade rõ rệt cho Episode 2 (tối hơn, giảm bão hoà, lạnh hơn) để khác hẳn Episode 1.</t>
         </is>
       </c>
     </row>
@@ -4655,7 +5006,12 @@
       </c>
       <c r="J71" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not a bug</t>
+        </is>
+      </c>
+      <c r="K71" s="12" t="inlineStr">
+        <is>
+          <t>Đi luồng thật (375 và 430): sau tin nhắn 1, counter hiển thị "Free preview · 1 message left". Lỗi chỉ do deep-jump seed data.</t>
         </is>
       </c>
     </row>
@@ -4705,7 +5061,12 @@
       </c>
       <c r="J72" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K72" s="12" t="inlineStr">
+        <is>
+          <t>Ở màn thấp (&lt;=700px) reply chip xuống dòng (wrap) thay vì hàng cuộn ẩn; cả 3 chip hiển thị đủ trong 375px.</t>
         </is>
       </c>
     </row>
@@ -4755,7 +5116,12 @@
       </c>
       <c r="J73" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not a bug</t>
+        </is>
+      </c>
+      <c r="K73" s="12" t="inlineStr">
+        <is>
+          <t>Luồng thật (kể cả bấm nhanh): toast hết hạn trước khi sang Intro 10, không đè headline/logo; lỗi do deep-jump liên tiếp. Vẫn gia cố: toast bị xoá khi đổi màn, giới hạn bề ngang và đặt dưới header chat.</t>
         </is>
       </c>
     </row>
@@ -4805,7 +5171,12 @@
       </c>
       <c r="J74" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K74" s="12" t="inlineStr">
+        <is>
+          <t>Sticky bar có nền đặc + viền trên; hiện bất cứ khi nào không có nút CTA của plan block trong màn hình (nên first view 375 và 430 đều có giá + Unlock Episode 3); thêm padding cuối trang để không che nội dung cuối.</t>
         </is>
       </c>
     </row>
@@ -4855,7 +5226,12 @@
       </c>
       <c r="J75" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K75" s="12" t="inlineStr">
+        <is>
+          <t>Xoá hẳn màn last_chance_offer (view, SCREENS, OFFER_ID, action offerbuy/offerno) và CONFIG.offer chứa {{offer_price}}; deep-jump #s=99 không mở được nữa. ff_engine_build vẫn build OK, checkout không đổi.</t>
         </is>
       </c>
     </row>

</xml_diff>